<commit_message>
cleaned up the code.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Riddh\OneDrive\Desktop\CapG\AIVS-JAVA\MCP\FinalCapstoneProject\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Riddh\OneDrive\Desktop\CapG\AIVS-JAVA\MCP\CapstoneProject\FinalCapstoneProject\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DA9CBB-F945-4F7B-A2AD-8A79160CC9D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10506B3F-6622-4D6C-99A9-2582431A107F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="100">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -315,9 +315,6 @@
   </si>
   <si>
     <t>DELETE_NOTE</t>
-  </si>
-  <si>
-    <t>INVALID_NOTE_ID</t>
   </si>
   <si>
     <t>GET_NOTES</t>
@@ -1351,7 +1348,7 @@
         <v>400</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1391,7 +1388,7 @@
         <v>400</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1426,14 +1423,14 @@
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="2" t="s">
-        <v>95</v>
+      <c r="F8" s="2">
+        <v>25</v>
       </c>
       <c r="G8" s="2">
         <v>401</v>
       </c>
       <c r="H8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1441,7 +1438,7 @@
         <v>81</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -1451,7 +1448,7 @@
         <v>401</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1459,7 +1456,7 @@
         <v>82</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -1469,7 +1466,7 @@
         <v>401</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>